<commit_message>
Optimizasyon yapıldı hatalar giderildi
</commit_message>
<xml_diff>
--- a/backtest_sonuclari.xlsx
+++ b/backtest_sonuclari.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9118.370000000001</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>1.85</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>71.73999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -488,111 +488,35 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-442.27</v>
+        <v>5219.93</v>
       </c>
       <c r="C3" t="n">
-        <v>12.77</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>165</v>
+        <v>146</v>
       </c>
       <c r="E3" t="n">
-        <v>26.06</v>
+        <v>32.19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HALKB</t>
+          <t>THYAO</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7930.25</v>
+        <v>2693.13</v>
       </c>
       <c r="C4" t="n">
-        <v>5.44</v>
+        <v>18.17</v>
       </c>
       <c r="D4" t="n">
-        <v>50</v>
+        <v>201</v>
       </c>
       <c r="E4" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ISCTR</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>8671.07</v>
-      </c>
-      <c r="C5" t="n">
-        <v>22.22</v>
-      </c>
-      <c r="D5" t="n">
-        <v>274</v>
-      </c>
-      <c r="E5" t="n">
-        <v>31.75</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>THYAO</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>20518.91</v>
-      </c>
-      <c r="C6" t="n">
-        <v>17.66</v>
-      </c>
-      <c r="D6" t="n">
-        <v>252</v>
-      </c>
-      <c r="E6" t="n">
-        <v>39.68</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>TUPRS</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>8058.73</v>
-      </c>
-      <c r="C7" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="D7" t="n">
-        <v>36</v>
-      </c>
-      <c r="E7" t="n">
-        <v>58.33</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>VAKBN</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>-172.83</v>
-      </c>
-      <c r="C8" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="D8" t="n">
-        <v>11</v>
-      </c>
-      <c r="E8" t="n">
-        <v>18.18</v>
+        <v>32.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>